<commit_message>
chore: WBS 자동 갱신 (2026-08-26)
</commit_message>
<xml_diff>
--- a/deliverables/plan/wbs.xlsx
+++ b/deliverables/plan/wbs.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="WBS" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -447,7 +447,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>17%</t>
+          <t>16%</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -457,7 +457,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>48%</t>
+          <t>45%</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1089,7 +1089,7 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1775,7 +1775,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>48%</t>
+          <t>45%</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">

</xml_diff>

<commit_message>
chore: WBS 자동 갱신 (2026-08-31)
</commit_message>
<xml_diff>
--- a/deliverables/plan/wbs.xlsx
+++ b/deliverables/plan/wbs.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="WBS" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -447,7 +447,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>17%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -457,7 +457,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -555,7 +555,7 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>48%</t>
+          <t>61%</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -582,12 +582,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>A3 평가</t>
+          <t>A1 정책 학습</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>[작업] RoboGauge 공개 정책 4종: 우리 평가에 붙이기</t>
+          <t>[작업] 실패 지형 5종 담당을 정한다</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -596,11 +596,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -608,15 +608,19 @@
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>48%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -638,36 +642,36 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>A3 평가</t>
+          <t>A1 정책 학습</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>[평가 체계]</t>
+          <t>[작업] 레일즈 MuJoCo 사전 측정과 Isaac 스윕 설계</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MVP · 중간발표</t>
+          <t>A-정책</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -677,68 +681,72 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>vfxpedia</t>
+          <t>maengu86</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>deliverables/midterm/generalization-report.md</t>
+          <t>deliverables/midterm/policy-metrics.md</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>foothold-go2</t>
+          <t>foothold-lab</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>A4 트윈·렌더</t>
+          <t>A1 정책 학습</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>[작업] 에셋 팩 수령과 HDRI 렌더 테스트</t>
+          <t>[작업] RunPod에서 Isaac 험지 지형 headless 생성·확인 환경 확보</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MVP · 중간발표</t>
+          <t>A-정책</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>vfxpedia</t>
+          <t>less82</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>deliverables/midterm/generalization-report.md</t>
+          <t>deliverables/midterm/policy-metrics.md</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -750,27 +758,45 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>B1 항법</t>
+          <t>A1 정책 학습</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>[작업] ROS 2 학습자료 01·ROS 2 개발환경 구축 정리</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
+          <t>[작업] 험지 지형 종류 확장 및 난이도 파라미터화</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>A-정책</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>13</v>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -778,7 +804,11 @@
           <t>less82</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>deliverables/midterm/policy-metrics.md</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>foothold-lab</t>
@@ -788,35 +818,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>B1 항법</t>
+          <t>A1 정책 학습</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>[작업] ROS 2 학습자료 02·ROS 2 Python 프로그래밍 정리</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
+          <t>[작업] 테스트</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MVP · 중간발표</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>35</v>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>12%</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>less82</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr"/>
+          <t>maengu86</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>deliverables/midterm/generalization-report.md</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>foothold-lab</t>
@@ -826,24 +878,38 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>B1 항법</t>
+          <t>A1 정책 학습</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>[작업] ROS 2 학습자료 03·TF 좌표계와 RViz2 시각화 정리</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
+          <t>[작업] 실패 지형 gap: 진단 -&gt; 레시피 (임석헌)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MVP · 중간발표</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>34</v>
+      </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>9%</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
           <t>0%</t>
@@ -851,10 +917,14 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>less82</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr"/>
+          <t>IQ152</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>deliverables/midterm/generalization-report.md</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>foothold-lab</t>
@@ -864,24 +934,38 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>B2 인지</t>
+          <t>A1 정책 학습</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>[작업] CV 담당 단계별 계획과 실행 환경 문서 제출</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
+          <t>[작업] 실패 지형 rails: 진단 -&gt; 레시피 (맹라현)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MVP · 중간발표</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>34</v>
+      </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>9%</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
           <t>0%</t>
@@ -889,10 +973,14 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>less82</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr"/>
+          <t>maengu86</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>deliverables/midterm/generalization-report.md</t>
+        </is>
+      </c>
       <c r="L11" t="inlineStr">
         <is>
           <t>foothold-lab</t>
@@ -902,36 +990,36 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C1 기록</t>
+          <t>A1 정책 학습</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>[승격 검토] inbox/meang/20260825-park-mentoring.md</t>
+          <t>[작업] 실패 지형 stepping_stones: 진단 -&gt; 레시피 (오현민)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>A-정책</t>
+          <t>MVP · 중간발표</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>9%</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -941,12 +1029,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>vfxpedia</t>
+          <t>less82</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>deliverables/midterm/policy-metrics.md</t>
+          <t>deliverables/midterm/generalization-report.md</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -958,12 +1046,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C1 기록</t>
+          <t>A1 정책 학습</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>[작업] 도구 백과 — 우리가 쓰는 도구들을 그림과 함께</t>
+          <t>[작업] 실패 지형 pit: 진단 -&gt; 레시피 (이민우)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -972,11 +1060,11 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -987,7 +1075,7 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>9%</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -997,7 +1085,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>vfxpedia</t>
+          <t>lmw0207</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1014,36 +1102,36 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C2 운영</t>
+          <t>A1 정책 학습</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>[인프라] Vaultwarden 개통 + NAS 폴더 구조</t>
+          <t>[작업] 실패 지형 floating_ring: 진단 -&gt; 레시피 (오흥재)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>A-정책</t>
+          <t>MVP · 중간발표</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>48%</t>
+          <t>9%</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1058,7 +1146,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>deliverables/midterm/policy-metrics.md</t>
+          <t>deliverables/midterm/generalization-report.md</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1070,40 +1158,40 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C2 운영</t>
+          <t>A2 지형·씬 제작</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>[작업] 자동 분류 배선 시험 2</t>
+          <t>[작업] 파인튜닝 가능한 지형 조사</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>A-정책</t>
+          <t>MVP · 중간발표</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>12%</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1113,12 +1201,12 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>vfxpedia</t>
+          <t>maengu86</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>deliverables/midterm/policy-metrics.md</t>
+          <t>deliverables/midterm/generalization-report.md</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1130,21 +1218,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C2 운영</t>
+          <t>A3 평가</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>[운영]</t>
+          <t>[작업] RoboGauge 공개 정책 4종: 우리 평가에 붙이기</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>FINAL · 최종발표</t>
+          <t>A-정책</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>122</v>
+        <v>32</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1153,13 +1241,13 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>61%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1169,29 +1257,29 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>vfxpedia</t>
+          <t>vfxpedia,less82</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>deliverables/final/final-report.md</t>
+          <t>deliverables/midterm/policy-metrics.md</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>foothold-go2</t>
+          <t>foothold-lab</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>C2 운영</t>
+          <t>A3 평가</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>[작업] 우분투 전환 후 DDP 재측정</t>
+          <t>[평가 체계]</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1215,7 +1303,7 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>39%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1235,42 +1323,60 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>foothold-lab</t>
+          <t>foothold-go2</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>(미분류)</t>
+          <t>A4 트윈·렌더</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>[작업] 자동화 배선 테스트</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
+          <t>[작업] 에셋 팩 수령과 HDRI 렌더 테스트</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MVP · 중간발표</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>50</v>
+      </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>39%</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>deliverables/midterm/generalization-report.md</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>foothold-lab</t>
@@ -1280,25 +1386,25 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>(미분류)</t>
+          <t>B1 항법</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>[실험] 배선 테스트 - 담당자 자동 지정 확인</t>
+          <t>[작업] ROS 2 학습자료 01·ROS 2 개발환경 구축 정리</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -1309,38 +1415,38 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>vfxpedia</t>
+          <t>less82</t>
         </is>
       </c>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>foothold-go2</t>
+          <t>foothold-lab</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>(미분류)</t>
+          <t>B1 항법</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>[작업] 협업 규칙 문서 초안 작성</t>
+          <t>[작업] ROS 2 학습자료 02·ROS 2 Python 프로그래밍 정리</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
@@ -1351,7 +1457,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>vfxpedia</t>
+          <t>less82</t>
         </is>
       </c>
       <c r="K20" t="inlineStr"/>
@@ -1364,25 +1470,25 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>(미분류)</t>
+          <t>B1 항법</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>[작업] 휘발 방지 — 결정 로그·검증 기록·재개 지점 문서화</t>
+          <t>[작업] ROS 2 학습자료 03·TF 좌표계와 RViz2 시각화 정리</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -1393,7 +1499,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>vfxpedia</t>
+          <t>less82</t>
         </is>
       </c>
       <c r="K21" t="inlineStr"/>
@@ -1406,39 +1512,53 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>(미분류)</t>
+          <t>B2 인지</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>[작업] 협업 규칙 COLLAB.md 작성 + collab.html 게시</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
+          <t>[작업] CV 담당 단계별 계획과 실행 환경 문서 제출</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>NAV · 실기 항법</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>74</v>
+      </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr"/>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>7%</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>vfxpedia</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr"/>
+          <t>less82</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>deliverables/final/nav-report.md</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>foothold-lab</t>
@@ -1448,36 +1568,32 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>(미분류)</t>
+          <t>C1 기록</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>[막힘] 사이트 5개 페이지 다크모드 미지원</t>
+          <t>[작업] 노션 프로젝트 기획 정리</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>vfxpedia</t>
+          <t>lmw0207</t>
         </is>
       </c>
       <c r="K23" t="inlineStr"/>
@@ -1490,25 +1606,25 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>(미분류)</t>
+          <t>C1 기록</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>[테스트] done date 자동 기입 검증</t>
+          <t>[작업] 저수준 이전·증류 잔재 정리 · 8/19 에 뺀 목표가 본문에 살아 있다</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -1532,31 +1648,41 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>(미분류)</t>
+          <t>C1 기록</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>[테스트] sub-issue 자동 연결 검증</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
+          <t>[승격 검토] inbox/meang/20260825-park-mentoring.md</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>A-정책</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>18</v>
+      </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr"/>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>29%</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1564,7 +1690,11 @@
           <t>vfxpedia</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>deliverables/midterm/policy-metrics.md</t>
+        </is>
+      </c>
       <c r="L25" t="inlineStr">
         <is>
           <t>foothold-lab</t>
@@ -1574,31 +1704,41 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>(미분류)</t>
+          <t>C1 기록</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>[테스트] 루프 차단 후 sub-issue 재검증</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
+          <t>[작업] 도구 백과 · 우리가 쓰는 도구들을 그림과 함께</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>MVP · 중간발표</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>53</v>
+      </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr"/>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>42%</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1606,7 +1746,11 @@
           <t>vfxpedia</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>deliverables/midterm/generalization-report.md</t>
+        </is>
+      </c>
       <c r="L26" t="inlineStr">
         <is>
           <t>foothold-lab</t>
@@ -1616,31 +1760,41 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>(미분류)</t>
+          <t>C1 기록</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>[실측] WS: DDP 판정 · 1,500 완주 · 평가 기준선 86.7% · 난이도 곡선</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
+          <t>[작업] 기술 레퍼런스 허브 신설 (허브 6번째)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>MVP · 중간발표</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>34</v>
+      </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr"/>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>9%</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -1648,7 +1802,11 @@
           <t>vfxpedia</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>deliverables/midterm/generalization-report.md</t>
+        </is>
+      </c>
       <c r="L27" t="inlineStr">
         <is>
           <t>foothold-lab</t>
@@ -1658,39 +1816,53 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>(미분류)</t>
+          <t>C1 기록</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>[웹] 연구 페이지 시각화: 이미지 15장 · 영상 재생 · 썸네일 · NEW 배지 · em dash 관문</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
+          <t>[작업] foothold-wiki 흡수 · 한 곳으로 모은다</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>MVP · 중간발표</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>34</v>
+      </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>9%</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>vfxpedia</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr"/>
+          <t>less82</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>deliverables/midterm/generalization-report.md</t>
+        </is>
+      </c>
       <c r="L28" t="inlineStr">
         <is>
           <t>foothold-lab</t>
@@ -1700,31 +1872,41 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>(미분류)</t>
+          <t>C1 기록</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>[승격 검토] inbox/oh/20260814-pipeline-test.md</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
+          <t>[작업] 허브 안 표현 재설계 · 위에서 아래로 흐르는 목록을 바꾼다</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>MVP · 중간발표</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>34</v>
+      </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr"/>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>9%</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -1732,7 +1914,11 @@
           <t>vfxpedia</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>deliverables/midterm/generalization-report.md</t>
+        </is>
+      </c>
       <c r="L29" t="inlineStr">
         <is>
           <t>foothold-lab</t>
@@ -1742,31 +1928,41 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>(미분류)</t>
+          <t>C1 기록</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>[승격 검토] inbox/lim/20260822-베이스라인 모델의 간단한 미경험 험지 성능 측정.md</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
+          <t>[작업] 사이트 온톨로지 정의 (무엇이 무엇의 상위인가)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>MVP · 중간발표</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>34</v>
+      </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr"/>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>9%</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -1774,7 +1970,11 @@
           <t>vfxpedia</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>deliverables/midterm/generalization-report.md</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>foothold-lab</t>
@@ -1784,25 +1984,25 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>(미분류)</t>
+          <t>C2 운영</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>[승격 검토] inbox/meang/20260818-rough-terrain-rl-study.md</t>
+          <t>[작업] 조선대 저장소 이력 소실 · 실습 zip 4종을 잃었다</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
@@ -1826,31 +2026,27 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>(미분류)</t>
+          <t>C2 운영</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>[작업] 자동 분류 배선 시험</t>
+          <t>[작업] 강의 저장소 감시가 알림만 한다. 미러까지 하게</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
+      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -1868,58 +2064,1608 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>C2 운영</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>[작업] v2.0.0 적용 완료 점검 · 여덟 가지를 실측으로 확인한다</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>C2 운영</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>[작업] PRD-WEB 정렬 패스 · 기준 한 장대로 전 화면을 맞춘다</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>C2 운영</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>[작업] 표지를 타겟 기준으로 재구성 · 온톨로지의 마지막 축을 쓴다</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>C2 운영</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>[인프라] Vaultwarden 개통 + NAS 폴더 구조</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>A-정책</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>32</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>61%</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>deliverables/midterm/policy-metrics.md</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>C2 운영</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>[작업] 자동 분류 배선 시험 2</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>A-정책</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>18</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>29%</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>deliverables/midterm/policy-metrics.md</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>C2 운영</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>[작업] RunPod 네트워크 볼륨 개설과 팀 폴더 구조 표준화</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>A-정책</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>13</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>less82</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>deliverables/midterm/policy-metrics.md</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>C2 운영</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>[운영]</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>FINAL · 최종발표</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>122</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2026-12-11</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>deliverables/final/final-report.md</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>foothold-go2</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>C2 운영</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>[작업] 우분투 전환 후 DDP 재측정</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>MVP · 중간발표</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>50</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>39%</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>deliverables/midterm/generalization-report.md</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>C2 운영</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>[작업] 일정 시스템 구현 (8/26 설계안이 통째로 증발했다)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>MVP · 중간발표</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>34</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>9%</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>deliverables/midterm/generalization-report.md</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>C2 운영</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>[작업] NEW 배지가 허브에서는 안 뜬다 (설계 재정비)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>MVP · 중간발표</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>34</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>9%</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>deliverables/midterm/generalization-report.md</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>C2 운영</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>[작업] 브랜드·테마 일관성: 전역바 로고가 정본이 아니다</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>MVP · 중간발표</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>34</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>9%</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>deliverables/midterm/generalization-report.md</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>C2 운영</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>[작업] WBS 자동 생성 결과가 웹에 도달하지 않는다</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>기획발표</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>(미분류)</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>[작업] 자동화 배선 테스트</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>[실험] 배선 테스트 - 담당자 자동 지정 확인</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>foothold-go2</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>[작업] 협업 규칙 문서 초안 작성</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>[작업] 휘발 방지 · 결정 로그·검증 기록·재개 지점 문서화</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>[작업] 협업 규칙 COLLAB.md 작성 + collab.html 게시</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>[막힘] 사이트 5개 페이지 다크모드 미지원</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>[테스트] done date 자동 기입 검증</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>[테스트] sub-issue 자동 연결 검증</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>[테스트] 루프 차단 후 sub-issue 재검증</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>[실측] WS: DDP 판정 · 1,500 완주 · 평가 기준선 86.7% · 난이도 곡선</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>[웹] 연구 페이지 시각화: 이미지 15장 · 영상 재생 · 썸네일 · NEW 배지 · em dash 관문</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>[승격 검토] inbox/oh/20260814-pipeline-test.md</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>[승격 검토] inbox/lim/20260822-베이스라인 모델의 간단한 미경험 험지 성능 측정.md</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>[승격 검토] inbox/meang/20260818-rough-terrain-rl-study.md</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>[작업] 자동 분류 배선 시험</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>[승격 검토] inbox/oh/20260826-ros2-01-개발환경구축.md</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>[주간] W35 팀 목표 (8/24~8/30)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>vfxpedia,less82,lmw0207,IQ152,maengu86</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>[주간] W36 오흥재 개인 목표</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>[주간] W36 맹라현 개인 목표</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>maengu86</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>[주간] W36 오현민 개인 목표</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>less82</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>[주간] W36 임석헌 개인 목표</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>IQ152</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>[주간] W36 이민우 개인 목표</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>lmw0207</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
         <is>
           <t>[8/13] 조선대 방문: FIELD-CHECK 수행</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C67" t="inlineStr">
         <is>
           <t>A-정책</t>
         </is>
       </c>
-      <c r="D33" t="n">
+      <c r="D67" t="n">
         <v>32</v>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E67" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F67" t="inlineStr">
         <is>
           <t>2026-09-12</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G67" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>48%</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>61%</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>vfxpedia</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>vfxpedia</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
         <is>
           <t>deliverables/midterm/policy-metrics.md</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr">
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>foothold-lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>(미분류)</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>[주간] W36 팀 목표 (8/31~9/6) · 기획발표 주</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>기획발표</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>vfxpedia,less82,lmw0207,IQ152,maengu86</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr">
         <is>
           <t>foothold-lab</t>
         </is>

</xml_diff>

<commit_message>
일정 확정 반영 (팀장 10/12): SIM 11/7 · NAV 11/30 · FINAL 12/7 (실제 발표 12/9 또는 12/10 · 12/11 수료식)
D-Day 띠 · 산출물 관문 · WBS 생성기 · 이슈 폼 · 분류 자동화 · WORKFLOW · COLLAB · DECISIONS · AGENTS.
GitHub 마일스톤: SIM 새로 만듦 (11/7) · NAV 11/30 · FINAL 12/7.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/plan/wbs.xlsx
+++ b/deliverables/plan/wbs.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="WBS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5062,7 +5062,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -5071,13 +5071,13 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>7%</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5564,7 +5564,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -5573,13 +5573,13 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>2026-11-07</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -5620,7 +5620,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -5629,13 +5629,13 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>2026-11-07</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -5676,7 +5676,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -5685,7 +5685,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>2026-11-07</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -5695,7 +5695,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>64%</t>
+          <t>49%</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -5736,7 +5736,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -5745,13 +5745,13 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>2026-11-07</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6582,7 +6582,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -6591,7 +6591,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -7954,7 +7954,7 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -7963,7 +7963,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>2026-11-07</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -7973,7 +7973,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>19%</t>
+          <t>11%</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -9982,7 +9982,7 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -9991,7 +9991,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
@@ -10001,7 +10001,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>52%</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -10042,7 +10042,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -10051,7 +10051,7 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
@@ -10102,7 +10102,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -10111,7 +10111,7 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="G176" t="inlineStr"/>
@@ -10158,7 +10158,7 @@
         </is>
       </c>
       <c r="D177" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -10167,13 +10167,13 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="G177" t="inlineStr"/>
       <c r="H177" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>7%</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -11994,7 +11994,7 @@
         </is>
       </c>
       <c r="D208" t="n">
-        <v>31</v>
+        <v>54</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -12003,13 +12003,13 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>2026-11-07</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="G208" t="inlineStr"/>
       <c r="H208" t="inlineStr">
         <is>
-          <t>13%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">

</xml_diff>

<commit_message>
일정 확정 반영: SIM 11/7 · NAV 11/30 · FINAL 12/7 (팀장 10/12) (#549)
* 일정 확정 반영 (팀장 10/12): SIM 11/7 · NAV 11/30 · FINAL 12/7 (실제 발표 12/9 또는 12/10 · 12/11 수료식)

D-Day 띠 · 산출물 관문 · WBS 생성기 · 이슈 폼 · 분류 자동화 · WORKFLOW · COLLAB · DECISIONS · AGENTS.
GitHub 마일스톤: SIM 새로 만듦 (11/7) · NAV 11/30 · FINAL 12/7.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

* 일정 확정 반영: 표지 «현 단계 · 다음 마일스톤» 목록 · 「12/10」 폐기 규칙 철회 (팀장 10/12 · 실제 발표 12/9 또는 12/10)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

---------

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/plan/wbs.xlsx
+++ b/deliverables/plan/wbs.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="WBS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5062,7 +5062,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -5071,13 +5071,13 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>7%</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5564,7 +5564,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -5573,13 +5573,13 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>2026-11-07</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -5620,7 +5620,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -5629,13 +5629,13 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>2026-11-07</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -5676,7 +5676,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -5685,7 +5685,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>2026-11-07</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -5695,7 +5695,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>64%</t>
+          <t>49%</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -5736,7 +5736,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -5745,13 +5745,13 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>2026-11-07</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6582,7 +6582,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -6591,7 +6591,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -7954,7 +7954,7 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -7963,7 +7963,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>2026-11-07</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -7973,7 +7973,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>19%</t>
+          <t>11%</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -9982,7 +9982,7 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -9991,7 +9991,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
@@ -10001,7 +10001,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>52%</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -10042,7 +10042,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -10051,7 +10051,7 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
@@ -10102,7 +10102,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -10111,7 +10111,7 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="G176" t="inlineStr"/>
@@ -10158,7 +10158,7 @@
         </is>
       </c>
       <c r="D177" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -10167,13 +10167,13 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="G177" t="inlineStr"/>
       <c r="H177" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>7%</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -11994,7 +11994,7 @@
         </is>
       </c>
       <c r="D208" t="n">
-        <v>31</v>
+        <v>54</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -12003,13 +12003,13 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>2026-11-07</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="G208" t="inlineStr"/>
       <c r="H208" t="inlineStr">
         <is>
-          <t>13%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">

</xml_diff>